<commit_message>
Fix Status Summary chart labels 3.
</commit_message>
<xml_diff>
--- a/Sales_Pipeline_Lead_Management.xlsx
+++ b/Sales_Pipeline_Lead_Management.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d5d8c1100fa95943/Desktop/Sales Pipeline and Lead Management System/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zoya1\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_C6E2D41AC193ECEA17AC776416BE51DD9879F044" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{66C129C5-C875-4C7C-923F-E7585F356D9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -861,7 +861,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-2514-4348-BCE5-D5ACEC3A8556}"/>
+              <c16:uniqueId val="{00000000-2511-497C-9408-4ED213708690}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1009,25 +1009,6 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </c:spPr>
-          <c:dLbls>
-            <c:spPr>
-              <a:noFill/>
-              <a:ln>
-                <a:noFill/>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-            <c:showLegendKey val="1"/>
-            <c:showVal val="1"/>
-            <c:showCatName val="1"/>
-            <c:showSerName val="1"/>
-            <c:showPercent val="1"/>
-            <c:showBubbleSize val="1"/>
-            <c:showLeaderLines val="1"/>
-            <c:extLst>
-              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
-            </c:extLst>
-          </c:dLbls>
           <c:cat>
             <c:strRef>
               <c:f>'Status Summary'!$A$4:$A$10</c:f>
@@ -1089,17 +1070,17 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-DEEB-47A9-8E7F-C5A47675928E}"/>
+              <c16:uniqueId val="{00000000-1341-41D9-97B8-AD5BF5A50382}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
         <c:dLbls>
-          <c:showLegendKey val="1"/>
-          <c:showVal val="1"/>
-          <c:showCatName val="1"/>
-          <c:showSerName val="1"/>
-          <c:showPercent val="1"/>
-          <c:showBubbleSize val="1"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
           <c:showLeaderLines val="1"/>
         </c:dLbls>
         <c:firstSliceAng val="0"/>
@@ -1108,7 +1089,7 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="r"/>
-      <c:overlay val="1"/>
+      <c:overlay val="0"/>
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>

</xml_diff>